<commit_message>
Updated with sst, ice and geomporhology layer details
</commit_message>
<xml_diff>
--- a/Environmnetal_data_metadata.xlsx
+++ b/Environmnetal_data_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://universitytasmania-my.sharepoint.com/personal/nicole_hill_utas_edu_au/Documents/UTAS_work/Projects/Benthic Diversity ARC/Analysis/ARC_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{C96BA8B1-3E59-468D-84B8-7B03779BC5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DB1BAFF7-804D-47A7-870C-EA7B0160B7C9}"/>
+  <xr:revisionPtr revIDLastSave="253" documentId="8_{C96BA8B1-3E59-468D-84B8-7B03779BC5AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3A2FE1E-90E4-4139-9D39-EEB0D6B22CFE}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2664" windowWidth="30960" windowHeight="12612" xr2:uid="{37A04AC2-0244-4B87-B563-6F6FD289412D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="41496" windowHeight="17496" xr2:uid="{37A04AC2-0244-4B87-B563-6F6FD289412D}"/>
   </bookViews>
   <sheets>
     <sheet name="BioMAS environmental Metadata" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="143">
   <si>
     <t>Variable</t>
   </si>
@@ -58,9 +58,6 @@
     <t>Bathymetry</t>
   </si>
   <si>
-    <t>Slope</t>
-  </si>
-  <si>
     <t>TPI5</t>
   </si>
   <si>
@@ -91,33 +88,6 @@
     <t>Seafloor temperatue</t>
   </si>
   <si>
-    <t>500m_shelf_waom2k_seafloorcurrents.Rdata</t>
-  </si>
-  <si>
-    <t>500m_shelf_waom2k_seafloortemperature.Rdata</t>
-  </si>
-  <si>
-    <t>500m_shelf_NPP_Cafe_filled_SummerAverage.Rdata</t>
-  </si>
-  <si>
-    <t>bathy_depth.Rdata</t>
-  </si>
-  <si>
-    <t>bathy_slope.Rdata</t>
-  </si>
-  <si>
-    <t>bathy_tpi.Rdata</t>
-  </si>
-  <si>
-    <t>bathy_tpi5.Rdata</t>
-  </si>
-  <si>
-    <t>bathy_tpi11.Rdata</t>
-  </si>
-  <si>
-    <t>Seaice</t>
-  </si>
-  <si>
     <t>m/s2</t>
   </si>
   <si>
@@ -139,15 +109,6 @@
     <t>Chla Autumn</t>
   </si>
   <si>
-    <t>Circumpolar_EnvData_ChlA_spring.Rdata</t>
-  </si>
-  <si>
-    <t>Circumpolar_EnvData_ChlA_summer.Rdata</t>
-  </si>
-  <si>
-    <t>Circumpolar_EnvData_ChlA_autumn.Rdata</t>
-  </si>
-  <si>
     <t>File name</t>
   </si>
   <si>
@@ -160,21 +121,12 @@
     <t>Average chla between 21 Mar and 21 Jun (2002-2020)</t>
   </si>
   <si>
-    <t>Surface temperature (OISST)</t>
-  </si>
-  <si>
     <t>fronts/ ssh? (satellite)</t>
   </si>
   <si>
     <t>Bottom salinity (Woam2k?)</t>
   </si>
   <si>
-    <t>O2 (CARS 2009)</t>
-  </si>
-  <si>
-    <t>Silicate (CARS 2009)</t>
-  </si>
-  <si>
     <t>C/N/O2- B-SOSE</t>
   </si>
   <si>
@@ -220,12 +172,6 @@
     <t>distance to shelf break</t>
   </si>
   <si>
-    <t>Currently not working?- look at VM &amp; raadtools.Nic</t>
-  </si>
-  <si>
-    <t>to extract on VM &amp; raadtools- Nic</t>
-  </si>
-  <si>
     <t>to extract on VM &amp; raadtools- NIc</t>
   </si>
   <si>
@@ -241,20 +187,290 @@
     <t>geomorphology</t>
   </si>
   <si>
-    <t>extract from AADC- Nic</t>
-  </si>
-  <si>
     <t>Chase down which model would be best for region  and see!</t>
   </si>
   <si>
     <t>Almost there!- Jan</t>
+  </si>
+  <si>
+    <t>OISST via raadtools</t>
+  </si>
+  <si>
+    <t>SST mean</t>
+  </si>
+  <si>
+    <t>sst_mean</t>
+  </si>
+  <si>
+    <t>sst_sd</t>
+  </si>
+  <si>
+    <t>Average SST between 1 Jan 2002 and 31 Dec 2020</t>
+  </si>
+  <si>
+    <t>Degrees C</t>
+  </si>
+  <si>
+    <t>SST variability</t>
+  </si>
+  <si>
+    <t>SST summer mean</t>
+  </si>
+  <si>
+    <t>SST summer variability</t>
+  </si>
+  <si>
+    <t>SST spring mean</t>
+  </si>
+  <si>
+    <t>SST spring variability</t>
+  </si>
+  <si>
+    <t>sst_sp_mean</t>
+  </si>
+  <si>
+    <t>sst_su_mean</t>
+  </si>
+  <si>
+    <t>sst_sp_sd</t>
+  </si>
+  <si>
+    <t>sst_su_sd</t>
+  </si>
+  <si>
+    <t>0.25 degree</t>
+  </si>
+  <si>
+    <t>Standard deviation of  SST between 1 Jan 2002 and 31 Dec 2020</t>
+  </si>
+  <si>
+    <t>Average spring (Sep-Nov) SST (2002-2020)</t>
+  </si>
+  <si>
+    <t>Standard deviation of spring (Sep-Nov) SST (2002-2020)</t>
+  </si>
+  <si>
+    <t>Average summer (Dec-Feb) SST (2002-2020)</t>
+  </si>
+  <si>
+    <t>Standard deviation of summer (Dec-Feb) SST (2002-2020)</t>
+  </si>
+  <si>
+    <t>Most recent version from AP- need to wrangle-Nic</t>
+  </si>
+  <si>
+    <t>N/P/Si Bioracle??</t>
+  </si>
+  <si>
+    <t>O2/Si/P (CARS 2009)</t>
+  </si>
+  <si>
+    <t>Standard deviation in sea ice cover during summer (Dec- Feb) 2002-2020</t>
+  </si>
+  <si>
+    <t>Proportion of time ocean is covered by sea ice concentration of &gt;85%</t>
+  </si>
+  <si>
+    <t>Sea ice cover</t>
+  </si>
+  <si>
+    <t>Sea ice summer mean</t>
+  </si>
+  <si>
+    <t>Sea ice summer variability</t>
+  </si>
+  <si>
+    <t>Mean sea ice cover during summer (Dec- Feb) 2002-2020</t>
+  </si>
+  <si>
+    <t>Sea ice summer max</t>
+  </si>
+  <si>
+    <t>Max sea ice cover during summer (Dec- Feb) 2002-2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>geomorph</t>
+  </si>
+  <si>
+    <t>categorical</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
+  <si>
+    <t>Hand digitised polygons converted to 500 m raster</t>
+  </si>
+  <si>
+    <t>http://dx.doi.org/10.4225/25/5b289b3bc07af</t>
+  </si>
+  <si>
+    <t>Geomorpohological categories</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_Gemorphology</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_ChlA_autumn</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_ChlA_summer</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_ChlA_spring</t>
+  </si>
+  <si>
+    <t>500m_shelf_waom2k_seafloortemperature</t>
+  </si>
+  <si>
+    <t>500m_shelf_waom2k_seafloorcurrents</t>
+  </si>
+  <si>
+    <t>500m_shelf_NPP_Cafe_filled_SummerAverage</t>
+  </si>
+  <si>
+    <t>bathy_tpi11</t>
+  </si>
+  <si>
+    <t>bathy_tpi5</t>
+  </si>
+  <si>
+    <t>bathy_tpi</t>
+  </si>
+  <si>
+    <t>bathy_slope</t>
+  </si>
+  <si>
+    <t>bathy_depth</t>
+  </si>
+  <si>
+    <t>Sea ice spring mean</t>
+  </si>
+  <si>
+    <t>Sea ice spring variability</t>
+  </si>
+  <si>
+    <t>Mean sea ice cover during summer (Sep-Nov) 2002-2020</t>
+  </si>
+  <si>
+    <t>Standard deviation in sea ice cover during summer (Sep-Nov) 2002-2020</t>
+  </si>
+  <si>
+    <t>Max sea ice cover during summer  (Sep-Nov) 2 2002-2020</t>
+  </si>
+  <si>
+    <t>Sea ice spring max</t>
+  </si>
+  <si>
+    <t>ice_sp_mean</t>
+  </si>
+  <si>
+    <t>ice_sp_sd</t>
+  </si>
+  <si>
+    <t>ice_sp_max</t>
+  </si>
+  <si>
+    <t>ice_su_mean</t>
+  </si>
+  <si>
+    <t>ice_su_max</t>
+  </si>
+  <si>
+    <t>ice_su_sd</t>
+  </si>
+  <si>
+    <t>Sea ice mean</t>
+  </si>
+  <si>
+    <t>Sea ice variability</t>
+  </si>
+  <si>
+    <t>Sea ice max</t>
+  </si>
+  <si>
+    <t>ice_mean</t>
+  </si>
+  <si>
+    <t>ice_max</t>
+  </si>
+  <si>
+    <t>ice_sd</t>
+  </si>
+  <si>
+    <t>for all ice files- change of satellite between Oct 2011 and June 2012 where is missing data</t>
+  </si>
+  <si>
+    <t>Average ice cover across all months between 19th June 2002 and 31 Dec 2020</t>
+  </si>
+  <si>
+    <t>6.25 km</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_max"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_su_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_su_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_sp_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_sp_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_SST["sst_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_sp_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_sp_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_sp_max"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_su_mean"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_su_sd"]</t>
+  </si>
+  <si>
+    <t>Circumpolar_EnvData_500m_shelf_ice["ice_su_max"]</t>
+  </si>
+  <si>
+    <t>AMSR via raadtools</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>originally sterographic polar- bilinearly interpolated to 500m</t>
+  </si>
+  <si>
+    <t>originally WGS84 lat/long- reprojected and bilinearly interpolated to 500 m</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -298,6 +514,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -331,10 +561,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -344,8 +575,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -658,15 +895,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5F7C515A-C8AD-4B88-B018-D4662A000C62}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.5546875" customWidth="1"/>
     <col min="2" max="2" width="14.21875" customWidth="1"/>
-    <col min="3" max="3" width="45.6640625" customWidth="1"/>
-    <col min="4" max="4" width="50.5546875" customWidth="1"/>
-    <col min="7" max="8" width="21.5546875" customWidth="1"/>
-    <col min="9" max="9" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="58.77734375" customWidth="1"/>
+    <col min="4" max="4" width="54.109375" customWidth="1"/>
+    <col min="5" max="5" width="15.33203125" customWidth="1"/>
+    <col min="6" max="6" width="23.21875" customWidth="1"/>
+    <col min="7" max="7" width="21.5546875" customWidth="1"/>
+    <col min="8" max="8" width="47.21875" customWidth="1"/>
+    <col min="9" max="9" width="24.5546875" customWidth="1"/>
     <col min="10" max="10" width="14.44140625" style="6" customWidth="1"/>
   </cols>
   <sheetData>
@@ -675,13 +915,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>5</v>
@@ -693,13 +933,13 @@
         <v>4</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -707,266 +947,690 @@
         <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>21</v>
+        <v>102</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>84</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>23</v>
+        <v>100</v>
       </c>
       <c r="E4" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>24</v>
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>25</v>
+        <v>98</v>
       </c>
       <c r="E6" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>18</v>
+        <v>96</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="E9" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>65</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>25</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>94</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>35</v>
+        <v>92</v>
       </c>
       <c r="J12" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E13" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" t="s">
+        <v>52</v>
+      </c>
+      <c r="G13" t="s">
+        <v>67</v>
+      </c>
+      <c r="H13" t="s">
+        <v>142</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" t="s">
+        <v>68</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="E14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" t="s">
+        <v>52</v>
+      </c>
+      <c r="G14" t="s">
+        <v>67</v>
+      </c>
+      <c r="H14" t="s">
+        <v>142</v>
+      </c>
+      <c r="J14" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E15" t="s">
+        <v>57</v>
+      </c>
+      <c r="F15" t="s">
+        <v>52</v>
+      </c>
+      <c r="G15" t="s">
+        <v>67</v>
+      </c>
+      <c r="H15" t="s">
+        <v>142</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" t="s">
+        <v>65</v>
+      </c>
+      <c r="C16" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E16" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" t="s">
+        <v>52</v>
+      </c>
+      <c r="G16" t="s">
+        <v>67</v>
+      </c>
+      <c r="H16" t="s">
+        <v>142</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+      <c r="B17" t="s">
+        <v>64</v>
+      </c>
+      <c r="C17" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="E17" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" t="s">
+        <v>52</v>
+      </c>
+      <c r="G17" t="s">
+        <v>67</v>
+      </c>
+      <c r="H17" t="s">
+        <v>142</v>
+      </c>
+      <c r="J17" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="J16" s="6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" t="s">
+        <v>72</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="E18" t="s">
+        <v>57</v>
+      </c>
+      <c r="F18" t="s">
+        <v>52</v>
+      </c>
+      <c r="G18" t="s">
         <v>67</v>
       </c>
-      <c r="J17" s="6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>60</v>
+      <c r="H18" t="s">
+        <v>142</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>68</v>
+        <v>43</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>68</v>
+        <v>78</v>
+      </c>
+      <c r="C19" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="B20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="E20" t="s">
+        <v>140</v>
+      </c>
+      <c r="F20" t="s">
+        <v>139</v>
+      </c>
+      <c r="G20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H20" t="s">
+        <v>141</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A21" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C21" t="s">
+        <v>122</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" t="s">
+        <v>140</v>
+      </c>
+      <c r="F21" t="s">
+        <v>139</v>
+      </c>
+      <c r="G21" t="s">
+        <v>123</v>
+      </c>
+      <c r="H21" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A22" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="B22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C22" t="s">
+        <v>122</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="E22" t="s">
+        <v>140</v>
+      </c>
+      <c r="F22" t="s">
+        <v>139</v>
+      </c>
+      <c r="G22" t="s">
+        <v>123</v>
+      </c>
+      <c r="H22" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A23" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="B23" t="s">
+        <v>109</v>
+      </c>
+      <c r="C23" t="s">
+        <v>105</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="E23" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" t="s">
+        <v>139</v>
+      </c>
+      <c r="G23" t="s">
+        <v>123</v>
+      </c>
+      <c r="H23" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A24" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="B24" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" t="s">
+        <v>140</v>
+      </c>
+      <c r="F24" t="s">
+        <v>139</v>
+      </c>
+      <c r="G24" t="s">
+        <v>123</v>
+      </c>
+      <c r="H24" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B25" t="s">
+        <v>111</v>
+      </c>
+      <c r="C25" t="s">
+        <v>107</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" t="s">
+        <v>140</v>
+      </c>
+      <c r="F25" t="s">
+        <v>139</v>
+      </c>
+      <c r="G25" t="s">
+        <v>123</v>
+      </c>
+      <c r="H25" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" t="s">
+        <v>112</v>
+      </c>
+      <c r="C26" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" t="s">
+        <v>140</v>
+      </c>
+      <c r="F26" t="s">
+        <v>139</v>
+      </c>
+      <c r="G26" t="s">
+        <v>123</v>
+      </c>
+      <c r="H26" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" t="s">
+        <v>114</v>
+      </c>
+      <c r="C27" t="s">
+        <v>76</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" t="s">
+        <v>140</v>
+      </c>
+      <c r="F27" t="s">
+        <v>139</v>
+      </c>
+      <c r="G27" t="s">
+        <v>123</v>
+      </c>
+      <c r="H27" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="B28" t="s">
+        <v>113</v>
+      </c>
+      <c r="C28" t="s">
+        <v>83</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="E28" t="s">
+        <v>140</v>
+      </c>
+      <c r="F28" t="s">
+        <v>139</v>
+      </c>
+      <c r="G28" t="s">
+        <v>123</v>
+      </c>
+      <c r="H28" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="J30" s="6" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B31" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" t="s">
+        <v>90</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E31" t="s">
+        <v>86</v>
+      </c>
+      <c r="G31" t="s">
+        <v>87</v>
+      </c>
+      <c r="H31" t="s">
+        <v>88</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="J20" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="J22" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="J23" s="6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
+      <c r="J32" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="J24" s="6" t="s">
-        <v>70</v>
+      <c r="J33" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="J34" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J35" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="J38" s="6" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="I31" r:id="rId1" xr:uid="{48012E50-483A-45A3-8AFC-F0E5B49421FE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -984,19 +1648,19 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>3</v>

</xml_diff>